<commit_message>
feat: maestro persistente, trazabilidad y control de proceso (fase 2)
- maestro.json persistente con CRUD (POST/PUT/DELETE) y pestana editable
- manifiesto por corrida en runs/ con SHA-256, parametros y totales
- deteccion informativa de duplicados exactos y cobertura del rango declarado
- exportacion opcional de solo filas filtradas (sufijo _filtrado)
- factores 20..1 calculados con n/21 exacto (9 celdas corregidas en el baseline)
- elimina semanasPorAnio sin uso; agrega pruebas de duplicados y factores
- regenera Pelven_generado_2026.xlsx con el calculo exacto
</commit_message>
<xml_diff>
--- a/Pelven_generado_2026.xlsx
+++ b/Pelven_generado_2026.xlsx
@@ -10418,7 +10418,7 @@
         <v>214</v>
       </c>
       <c r="Q115" s="7">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="R115" s="7">
         <v>183</v>
@@ -11649,7 +11649,7 @@
         <v>515</v>
       </c>
       <c r="L129" s="7">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="M129" s="7">
         <v>460</v>
@@ -11786,7 +11786,7 @@
         <v>65</v>
       </c>
       <c r="AB130" s="7">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AC130" s="7">
         <v>22</v>
@@ -12005,7 +12005,7 @@
         <v>350</v>
       </c>
       <c r="L133" s="7">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="M133" s="7">
         <v>313</v>
@@ -14052,7 +14052,7 @@
         <v>477</v>
       </c>
       <c r="L156" s="7">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="M156" s="7">
         <v>426</v>
@@ -14319,7 +14319,7 @@
         <v>572</v>
       </c>
       <c r="L159" s="7">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="M159" s="7">
         <v>511</v>
@@ -14675,7 +14675,7 @@
         <v>426</v>
       </c>
       <c r="L163" s="7">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="M163" s="7">
         <v>381</v>
@@ -14764,7 +14764,7 @@
         <v>584</v>
       </c>
       <c r="L164" s="7">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="M164" s="7">
         <v>523</v>
@@ -15298,7 +15298,7 @@
         <v>388</v>
       </c>
       <c r="L170" s="7">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="M170" s="7">
         <v>347</v>

</xml_diff>